<commit_message>
docs(2.3+2.5/D1-D-2,D-3): 起草 ADR-007 权限矩阵 + ADR-008 数据层设计
- ADR-007(2.3): RBAC+按action鉴权+默认拒绝+多角色并集；4角色×全模块角色-权限矩阵，兼容 test-data ROLE_MATRIX 11 条契约；API 入口 requirePermission() 落地 3.4；跨租户平台超管暂缓阶段6；3 待拍板点
- ADR-008(2.5): 四层单向依赖，组件禁直连 mock/supabase，lib/data/* 唯一碰库+ctx+server-only，Repository 逐页切配合 3.5；铁律写入 CLAUDE.md
- 同步 ROADMAP(2.3/2.5→🔄 + 决策日志两行)、进度 Excel

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AIPaddle-项目进度管控.xlsx
+++ b/docs/AIPaddle-项目进度管控.xlsx
@@ -3534,12 +3534,12 @@
       </c>
       <c r="O27" s="45" t="inlineStr">
         <is>
-          <t>test-data ROLE_MATRIX</t>
+          <t>docs/adr/ADR-007-rbac-permission-model.md; test-data ROLE_MATRIX; TC-S0权限组</t>
         </is>
       </c>
       <c r="P27" s="46" t="inlineStr">
         <is>
-          <t>用例先行</t>
+          <t>ADR-007起草完成(2026-07-20)待拍板；RBAC+按action鉴权+默认拒绝+多角色并集；4角色x全模块矩阵(兼容ROLE_MATRIX 11条)；API入口requirePermission()落地3.4；平台超管暂缓阶段6；3待拍板点</t>
         </is>
       </c>
       <c r="Q27" s="45" t="inlineStr">
@@ -3621,10 +3621,14 @@
       </c>
       <c r="O28" s="47" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P28" s="48" t="n"/>
+          <t>docs/adr/ADR-008-data-access-layer.md</t>
+        </is>
+      </c>
+      <c r="P28" s="48" t="inlineStr">
+        <is>
+          <t>ADR-008起草完成(2026-07-20)待拍板；四层单向依赖(组件-&gt;API-&gt;lib/data-&gt;supabase)；组件禁直连mock/supabase；lib/data唯一碰库+ctx+server-only；Repository逐页切配合3.5；铁律入CLAUDE.md</t>
+        </is>
+      </c>
       <c r="Q28" s="47" t="inlineStr">
         <is>
           <t>—</t>

</xml_diff>

<commit_message>
docs(2.3+2.5/D1-D-2,D-3): 拍板 ADR-007 权限矩阵(补企业级上架审核) + ADR-008 数据层
- ADR-007 采纳并按 PRD 1.2/2.3/2.6 补齐统一上架审核流程：
  - PRD 业务角色↔4 技术角色映射；业务部门 AIBP=协同审批人
  - Agent/Skill/Workflow·Chatflow 三资产共用 draft→pending→published 状态机
  - 部门级 Admin/Auditor 单审；企业级仅 Admin 创建、Admin 必审 + 可指派 AIBP 协同双签
  - 矩阵新增 *:create:enterprise / *:review:cooperate 动作行
  - 已拍板：Auditor 不可 chat；平台超管暂缓阶段 6
- ADR-008 采纳：四层数据层单向依赖，铁律已入 CLAUDE.md
- ROADMAP 2.3/2.5→✅ + 决策日志转正；进度 Excel 同步

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AIPaddle-项目进度管控.xlsx
+++ b/docs/AIPaddle-项目进度管控.xlsx
@@ -3499,7 +3499,7 @@
       </c>
       <c r="H27" s="46" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="I27" s="45" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="P27" s="46" t="inlineStr">
         <is>
-          <t>ADR-007起草完成(2026-07-20)待拍板；RBAC+按action鉴权+默认拒绝+多角色并集；4角色x全模块矩阵(兼容ROLE_MATRIX 11条)；API入口requirePermission()落地3.4；平台超管暂缓阶段6；3待拍板点</t>
+          <t>ADR-007已拍板(2026-07-20)；RBAC+按action鉴权+默认拒绝+多角色并集；4角色x全模块矩阵；按PRD补齐统一上架审核：Agent/Skill/Workflow三资产共用draft-&gt;pending-&gt;published，部门级Admin/Auditor单审，企业级仅Admin创建+Admin必审+可指派AIBP协同双签；requirePermission()落地3.4；平台超管暂缓阶段6</t>
         </is>
       </c>
       <c r="Q27" s="45" t="inlineStr">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="H28" s="48" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>已完成</t>
         </is>
       </c>
       <c r="I28" s="47" t="inlineStr">
@@ -3626,7 +3626,7 @@
       </c>
       <c r="P28" s="48" t="inlineStr">
         <is>
-          <t>ADR-008起草完成(2026-07-20)待拍板；四层单向依赖(组件-&gt;API-&gt;lib/data-&gt;supabase)；组件禁直连mock/supabase；lib/data唯一碰库+ctx+server-only；Repository逐页切配合3.5；铁律入CLAUDE.md</t>
+          <t>ADR-008已拍板(2026-07-20)；四层单向依赖(组件-&gt;API-&gt;lib/data-&gt;supabase)；组件禁直连mock/supabase；lib/data唯一碰库+ctx+server-only；Repository逐页切配合3.5；铁律入CLAUDE.md</t>
         </is>
       </c>
       <c r="Q28" s="47" t="inlineStr">

</xml_diff>

<commit_message>
chore: close [0.7] server deployment - user verified
- User confirmed login via incognito at https://aipaddle.net
- ROADMAP.md 0.7 updated to ✅
- Excel progress updated
- GitHub Issue #52 closed

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AIPaddle-项目进度管控.xlsx
+++ b/docs/AIPaddle-项目进度管控.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📋 任务清单" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🚩 里程碑关口" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📝 决策日志" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⚠️ 问题台账" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51,7 +52,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -98,8 +99,13 @@
         <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -121,11 +127,55 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -185,6 +235,14 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,7 +623,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AIPaddle 项目进度仪表盘  ·  2026-07-20</t>
+          <t>AIPaddle 项目进度仪表盘  ·  2026-07-20（本次更新）</t>
         </is>
       </c>
     </row>
@@ -760,6 +818,9 @@
           <t>3.1 Seed 脚本已执行，Supabase 两租户五账号数据已写入</t>
         </is>
       </c>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="22" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
@@ -772,6 +833,9 @@
           <t>3.2 登录/注册/退出已实装，用户亲手验证登录成功</t>
         </is>
       </c>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="22" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
@@ -784,6 +848,9 @@
           <t>原型迁入 public/prototype/，根路径跳转逻辑已配置</t>
         </is>
       </c>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="22" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
@@ -796,6 +863,9 @@
           <t>0.7 服务器部署（aipaddle.net）：代码已部署，需亲手在线验证</t>
         </is>
       </c>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="22" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
@@ -808,6 +878,9 @@
           <t>#49/#50 Issue 标签仍显示「未开始」，需关闭并回填状态</t>
         </is>
       </c>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="22" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
@@ -820,6 +893,9 @@
           <t>[3.3] 租户上下文中间件 — 当前应执行任务</t>
         </is>
       </c>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1311,156 +1387,156 @@
       <c r="O7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>D1前</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>阶段0 环境</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>GitHub Issues 工作流（模板+标签+批量建卡）</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
-        <is>
-          <t>🔄 进行中</t>
-        </is>
-      </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="10" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>模板已入库；标签部分建立</t>
         </is>
       </c>
-      <c r="K8" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L8" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="17" t="inlineStr">
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M8" s="16" t="inlineStr">
         <is>
           <t>部分</t>
         </is>
       </c>
-      <c r="N8" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O8" s="10" t="inlineStr">
-        <is>
-          <t>标签体系已定义；批量建卡待做</t>
+      <c r="N8" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>GitHub Issues工作流：标签+模板+全量Issue已按ROADMAP v2.0重建（2026-07-20）</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>0.7</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>阶段0 环境</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>infra</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>服务器部署链路（43.173.99.218→aipaddle.net）</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>🔄 进行中</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>AI+Perry</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>0.2</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Issue#52；线上可访问</t>
         </is>
       </c>
-      <c r="K9" s="17" t="inlineStr">
+      <c r="K9" s="16" t="inlineStr">
         <is>
           <t>E2E冒烟</t>
         </is>
       </c>
-      <c r="L9" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M9" s="17" t="inlineStr">
+      <c r="L9" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M9" s="16" t="inlineStr">
         <is>
           <t>待验收</t>
         </is>
       </c>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="N9" s="16" t="inlineStr">
         <is>
           <t>P-GLB-01</t>
         </is>
       </c>
-      <c r="O9" s="10" t="inlineStr">
-        <is>
-          <t>代码已部署PM2，需用户亲手验证</t>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>隐私窗口登录验收通过（2026-07-20），Issue #52 关闭</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1548,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -1535,7 +1611,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O10" s="19" t="inlineStr"/>
+      <c r="O10" s="19" t="inlineStr">
+        <is>
+          <t>依赖0.7验收完成后执行；需Perry先在GitHub配置SSH_PRIVATE_KEY和SERVER_HOST两个Secret</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
@@ -1545,7 +1625,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1560,7 +1640,7 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>测试基建：Playwright已装；Vitest+RTL待做</t>
+          <t>测试基建：Playwright+Vitest+RTL已装；仅剩 0.9c 分支保护</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
@@ -1600,7 +1680,7 @@
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>部分通过</t>
+          <t>冒烟6条+单元7条全绿</t>
         </is>
       </c>
       <c r="N11" s="17" t="inlineStr">
@@ -1610,7 +1690,7 @@
       </c>
       <c r="O11" s="10" t="inlineStr">
         <is>
-          <t>0.9a完成；0.9b/c待做</t>
+          <t>0.9a✅Playwright 6条冒烟绿；0.9b✅Vitest+RTL装好(vitest.config+setup+test脚本),单元样例7条绿,CI启用单元测试步骤；待0.9c开main分支保护</t>
         </is>
       </c>
     </row>
@@ -1841,79 +1921,79 @@
       <c r="O15" s="8" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>阶段1 产品</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>docs</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>MVP首个闭环场景确认</t>
         </is>
       </c>
-      <c r="F16" s="17" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>🔄 进行中</t>
-        </is>
-      </c>
-      <c r="H16" s="17" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>Perry</t>
         </is>
       </c>
-      <c r="I16" s="10" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>确认 Agent 管理为第一条闭环</t>
         </is>
       </c>
-      <c r="K16" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L16" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M16" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N16" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O16" s="10" t="inlineStr">
-        <is>
-          <t>建议 Agent 管理；待用户拍板</t>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>MVP首个闭环=Agent管理（切片1），2026-07-20拍板，检测关口1放行</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2919,7 @@
       </c>
       <c r="O30" s="20" t="inlineStr">
         <is>
-          <t>⭐ 当前应执行任务</t>
+          <t>下一个待执行任务；依赖3.1/3.2</t>
         </is>
       </c>
     </row>
@@ -2914,7 +2994,11 @@
           <t>S0-PERM-01~06</t>
         </is>
       </c>
-      <c r="O31" s="19" t="inlineStr"/>
+      <c r="O31" s="19" t="inlineStr">
+        <is>
+          <t>依赖3.3</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="18" t="inlineStr">
@@ -2987,7 +3071,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O32" s="19" t="inlineStr"/>
+      <c r="O32" s="19" t="inlineStr">
+        <is>
+          <t>依赖3.3/3.4</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="18" t="inlineStr">
@@ -3060,7 +3148,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="O33" s="19" t="inlineStr"/>
+      <c r="O33" s="19" t="inlineStr">
+        <is>
+          <t>依赖0.7验收</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="18" t="inlineStr">
@@ -3133,7 +3225,11 @@
           <t>S0-ISO-*</t>
         </is>
       </c>
-      <c r="O34" s="19" t="inlineStr"/>
+      <c r="O34" s="19" t="inlineStr">
+        <is>
+          <t>检测关口3硬闸，必须全绿</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="15" t="inlineStr">
@@ -4123,12 +4219,12 @@
       </c>
       <c r="D2" s="17" t="inlineStr">
         <is>
-          <t>🔄 进行中</t>
+          <t>✅ 通过</t>
         </is>
       </c>
       <c r="E2" s="10" t="inlineStr">
         <is>
-          <t>Agent管理建议；待Perry拍板</t>
+          <t>Agent管理作为MVP首个闭环，2026-07-20拍板</t>
         </is>
       </c>
     </row>
@@ -4182,7 +4278,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>当前进行3.3</t>
+          <t>0.7已验收；下一步3.3租户中间件</t>
         </is>
       </c>
     </row>
@@ -4527,4 +4623,126 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>任务</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>问题描述</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>解决方案</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>负责方</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0.7 服务器部署</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>服务器无git pull能力（HTTPS无凭证），每次部署需手动rsync</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>等0.8 GitHub Actions上线后自动化解决</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>⚠️ 遗留</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AI（0.8完成后自动解决）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0.9a Playwright</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CI中测试步骤仍被注释，自动化测试未在CI运行</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.9c：启用ci.yml测试步骤+开main分支保护</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>⬜ 待处理</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>会话管理</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Supabase JWT Expiry仍为3600s（默认1h），24h硬限制可能被refresh token绕过</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>前往Supabase Dashboard→Auth→Configuration，将JWT expiry改为86400</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>⚠️ 需Perry操作</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Perry</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>